<commit_message>
Retirada da criação das tabelas no BD dos DAO's e repassada para o databaseInitializer e algumas correcoes no método de listar movimentações, alteração no processamentoService para ele usar o databaseInitializer, retirada do try em conexaoDAO e alteração da Main para ela usar o inicializarSistema do processamentoService.
</commit_message>
<xml_diff>
--- a/uploads/produtos.xlsx
+++ b/uploads/produtos.xlsx
@@ -364,7 +364,7 @@
         <v>150</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5</v>
@@ -387,7 +387,7 @@
         <v>350</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>5</v>
@@ -410,7 +410,7 @@
         <v>1200</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Atualiza logs e .gitignore
</commit_message>
<xml_diff>
--- a/uploads/produtos.xlsx
+++ b/uploads/produtos.xlsx
@@ -341,7 +341,7 @@
         <v>4500</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>3</v>
@@ -387,7 +387,7 @@
         <v>350</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>5</v>
@@ -410,7 +410,7 @@
         <v>1200</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>

</xml_diff>